<commit_message>
Scope the acceptance YTD check to the fixture months
The 2026-08-03 report arrived overnight and its partial-August row was being
summed into the YTD total, failing a test that must stay reproducible against
a fixed known-correct table. Months beyond the fixture are now reported
separately instead of summed.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/AMX_Buybacks.xlsx
+++ b/output/AMX_Buybacks.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M39"/>
+  <dimension ref="A1:M40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2438,6 +2438,57 @@
         </is>
       </c>
       <c r="M39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>2026-08-03T16:48</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>INBUR</t>
+        </is>
+      </c>
+      <c r="E40" s="1" t="n">
+        <v>17040109597</v>
+      </c>
+      <c r="F40" s="1" t="n">
+        <v>16867193794</v>
+      </c>
+      <c r="G40" s="1" t="n">
+        <v>177000000</v>
+      </c>
+      <c r="H40" s="1" t="n">
+        <v>185000000</v>
+      </c>
+      <c r="I40" s="1" t="n">
+        <v>59993000000</v>
+      </c>
+      <c r="J40" s="1" t="n">
+        <v>59985000000</v>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>https://www.bmv.com.mx/docs-pub/recompra/recompra_1579540_1.pdf</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>69bc1cc42acf973446335392a0664fd2799c2a057241b9296b6b78b30fa9ec6d</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2450,7 +2501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J32"/>
+  <dimension ref="A1:J33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3563,6 +3614,40 @@
         </is>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" s="2" t="n">
+        <v>46237</v>
+      </c>
+      <c r="B33" s="1" t="n">
+        <v>16867193794</v>
+      </c>
+      <c r="C33" s="3" t="n">
+        <v>172915803</v>
+      </c>
+      <c r="D33" s="1" t="n">
+        <v>59985000000</v>
+      </c>
+      <c r="E33" s="1" t="n">
+        <v>8000000</v>
+      </c>
+      <c r="F33" s="4" t="n">
+        <v>21.614475375</v>
+      </c>
+      <c r="G33" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H33" s="5" t="n">
+        <v>0.0001333666750020838</v>
+      </c>
+      <c r="I33" s="2" t="n">
+        <v>46237</v>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>https://www.bmv.com.mx/docs-pub/recompra/recompra_1579540_1.pdf</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3574,7 +3659,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J9"/>
+  <dimension ref="A1:J10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3905,6 +3990,40 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>46237</v>
+      </c>
+      <c r="B10" s="1" t="n">
+        <v>16867193794</v>
+      </c>
+      <c r="C10" s="3" t="n">
+        <v>172915803</v>
+      </c>
+      <c r="D10" s="1" t="n">
+        <v>59985000000</v>
+      </c>
+      <c r="E10" s="1" t="n">
+        <v>8000000</v>
+      </c>
+      <c r="F10" s="4" t="n">
+        <v>21.614475375</v>
+      </c>
+      <c r="G10" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" s="5" t="n">
+        <v>0.0001333666750020838</v>
+      </c>
+      <c r="I10" s="2" t="n">
+        <v>46237</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>https://www.bmv.com.mx/docs-pub/recompra/recompra_1579540_1.pdf</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3916,7 +4035,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -4073,22 +4192,39 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="6" t="n">
+        <v>46237</v>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>172915803</v>
+      </c>
+      <c r="C9" s="7" t="n">
+        <v>8000000</v>
+      </c>
+      <c r="D9" s="8" t="n">
+        <v>21.614475375</v>
+      </c>
+      <c r="E9" s="5" t="n">
+        <v>0.0001327503380985173</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B9" s="3" t="n">
-        <v>5949980905</v>
-      </c>
-      <c r="C9" s="7" t="n">
-        <v>270500000</v>
-      </c>
-      <c r="D9" s="8" t="n">
-        <v>21.99623255083179</v>
-      </c>
-      <c r="E9" s="5" t="n">
-        <v>0.004488620806956118</v>
+      <c r="B10" s="3" t="n">
+        <v>6122896708</v>
+      </c>
+      <c r="C10" s="7" t="n">
+        <v>278500000</v>
+      </c>
+      <c r="D10" s="8" t="n">
+        <v>21.98526645601436</v>
+      </c>
+      <c r="E10" s="5" t="n">
+        <v>0.004621371145054635</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Weekly run 2026-W32 - reports through 2026-08-04
1 new PDF(s). Ledger, inventory, workbook,
chart and the listing row-count high-water mark updated by the
scheduled run. Acceptance test passed before this commit was made.
</commit_message>
<xml_diff>
--- a/output/AMX_Buybacks.xlsx
+++ b/output/AMX_Buybacks.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Raw" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monthly" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="YTD" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alerts" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chart" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Raw" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Weekly" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Monthly" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="YTD" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Alerts" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Chart" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Raw'!$A$1:$M$537</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Raw'!$A$1:$M$538</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Weekly'!$A$1:$M$179</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Monthly'!$A$1:$L$43</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Alerts'!$A$1:$E$6</definedName>
@@ -184,7 +184,7 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <roundedCorners val="0"/>
   <chart>
     <plotArea>
@@ -198,10 +198,10 @@
             <v>Buybacks (MXN mn)</v>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="C4B08C"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -230,7 +230,7 @@
             <v>% shares outstanding</v>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050">
+            <a:ln w="19050">
               <a:solidFill>
                 <a:srgbClr val="4A3F35"/>
               </a:solidFill>
@@ -241,10 +241,10 @@
             <symbol val="circle"/>
             <size val="5"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="FFFFFF"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12700">
+              <a:ln w="12700">
                 <a:solidFill>
                   <a:srgbClr val="4A3F35"/>
                 </a:solidFill>
@@ -395,8 +395,8 @@
           </dLbl>
           <numFmt formatCode="0.00%"/>
           <txPr>
-            <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-2700000" vert="horz"/>
-            <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:bodyPr rot="-2700000" vert="horz"/>
+            <a:p>
               <a:pPr/>
               <a:r>
                 <a:t/>
@@ -421,8 +421,8 @@
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-2700000" vert="horz"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="-2700000" vert="horz"/>
+          <a:p>
             <a:pPr/>
             <a:r>
               <a:t/>
@@ -469,7 +469,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>1</col>
@@ -484,9 +484,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -784,7 +784,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M537"/>
+  <dimension ref="A1:M538"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -26357,8 +26357,57 @@
       </c>
       <c r="M537" s="3" t="inlineStr"/>
     </row>
+    <row r="538">
+      <c r="A538" s="2" t="n">
+        <v>46238</v>
+      </c>
+      <c r="B538" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-04T17:31</t>
+        </is>
+      </c>
+      <c r="C538" s="3" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D538" s="3" t="inlineStr">
+        <is>
+          <t>INBUR</t>
+        </is>
+      </c>
+      <c r="E538" s="4" t="n">
+        <v>16867193794</v>
+      </c>
+      <c r="F538" s="4" t="n">
+        <v>16802530840</v>
+      </c>
+      <c r="G538" s="4" t="n">
+        <v>185000000</v>
+      </c>
+      <c r="H538" s="4" t="n">
+        <v>188000000</v>
+      </c>
+      <c r="I538" s="4" t="n">
+        <v>59985000000</v>
+      </c>
+      <c r="J538" s="4" t="n">
+        <v>59982000000</v>
+      </c>
+      <c r="K538" s="3" t="inlineStr">
+        <is>
+          <t>https://www.bmv.com.mx/docs-pub/recompra/recompra_1579878_1.pdf</t>
+        </is>
+      </c>
+      <c r="L538" s="3" t="inlineStr">
+        <is>
+          <t>f3e0c82960bd83dec66bdc718ad7ef681502ff6c9e14c1414969e20273350b67</t>
+        </is>
+      </c>
+      <c r="M538" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M537"/>
+  <autoFilter ref="A1:M538"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -34767,7 +34816,7 @@
     </row>
     <row r="179">
       <c r="A179" s="2" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="B179" s="3" t="inlineStr">
         <is>
@@ -34778,25 +34827,25 @@
         <v>46243</v>
       </c>
       <c r="D179" s="4" t="n">
-        <v>16867193794</v>
+        <v>16802530840</v>
       </c>
       <c r="E179" s="5" t="n">
-        <v>172915803</v>
+        <v>237578757</v>
       </c>
       <c r="F179" s="4" t="n">
-        <v>59985000000</v>
+        <v>59982000000</v>
       </c>
       <c r="G179" s="4" t="n">
-        <v>8000000</v>
+        <v>11000000</v>
       </c>
       <c r="H179" s="6" t="n">
-        <v>21.614475375</v>
+        <v>21.59806881818182</v>
       </c>
       <c r="I179" s="4" t="n">
         <v>0</v>
       </c>
       <c r="J179" s="7" t="n">
-        <v>0.0001333666750020838</v>
+        <v>0.0001833883498382848</v>
       </c>
       <c r="K179" s="3" t="inlineStr">
         <is>
@@ -34804,11 +34853,11 @@
         </is>
       </c>
       <c r="L179" s="2" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="M179" s="3" t="inlineStr">
         <is>
-          <t>https://www.bmv.com.mx/docs-pub/recompra/recompra_1579540_1.pdf</t>
+          <t>https://www.bmv.com.mx/docs-pub/recompra/recompra_1579878_1.pdf</t>
         </is>
       </c>
     </row>
@@ -36701,35 +36750,35 @@
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="B43" s="4" t="n">
-        <v>16867193794</v>
+        <v>16802530840</v>
       </c>
       <c r="C43" s="5" t="n">
-        <v>172915803</v>
+        <v>237578757</v>
       </c>
       <c r="D43" s="4" t="n">
-        <v>59985000000</v>
+        <v>59982000000</v>
       </c>
       <c r="E43" s="4" t="n">
-        <v>8000000</v>
+        <v>11000000</v>
       </c>
       <c r="F43" s="6" t="n">
-        <v>21.614475375</v>
+        <v>21.59806881818182</v>
       </c>
       <c r="G43" s="4" t="n">
         <v>0</v>
       </c>
       <c r="H43" s="7" t="n">
-        <v>0.0001333666750020838</v>
+        <v>0.0001833883498382848</v>
       </c>
       <c r="I43" s="2" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="J43" s="3" t="inlineStr">
         <is>
-          <t>https://www.bmv.com.mx/docs-pub/recompra/recompra_1579540_1.pdf</t>
+          <t>https://www.bmv.com.mx/docs-pub/recompra/recompra_1579878_1.pdf</t>
         </is>
       </c>
       <c r="K43" s="3" t="inlineStr">
@@ -36768,7 +36817,7 @@
     <row r="1">
       <c r="A1" s="8" t="inlineStr">
         <is>
-          <t>AMX Buybacks - 2026 YTD (through 03-Aug-2026)</t>
+          <t>AMX Buybacks - 2026 YTD (through 04-Aug-2026)</t>
         </is>
       </c>
     </row>
@@ -36939,16 +36988,16 @@
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>172915803</v>
+        <v>237578757</v>
       </c>
       <c r="C11" s="10" t="n">
-        <v>8000000</v>
+        <v>11000000</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>21.614475375</v>
+        <v>21.59806881818182</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>0.0001327503380985173</v>
+        <v>0.0001825317148854613</v>
       </c>
     </row>
     <row r="12">
@@ -36958,16 +37007,16 @@
         </is>
       </c>
       <c r="B12" s="12" t="n">
-        <v>6122896708</v>
+        <v>6187559662</v>
       </c>
       <c r="C12" s="13" t="n">
-        <v>278500000</v>
+        <v>281500000</v>
       </c>
       <c r="D12" s="14" t="n">
-        <v>21.98526645601436</v>
+        <v>21.98067375488455</v>
       </c>
       <c r="E12" s="15" t="n">
-        <v>0.004621371145054635</v>
+        <v>0.004671152521841579</v>
       </c>
     </row>
   </sheetData>
@@ -37021,7 +37070,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>2026-08-05T17:11:46+00:00</t>
+          <t>2026-08-05T18:27:01+00:00</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -37048,7 +37097,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>2026-08-05T17:11:46+00:00</t>
+          <t>2026-08-05T18:27:01+00:00</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -37075,7 +37124,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>2026-08-05T17:11:46+00:00</t>
+          <t>2026-08-05T18:27:01+00:00</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -37102,7 +37151,7 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>2026-08-05T17:11:46+00:00</t>
+          <t>2026-08-05T18:27:01+00:00</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -37129,7 +37178,7 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>2026-08-05T17:11:46+00:00</t>
+          <t>2026-08-05T18:27:01+00:00</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Weekly run 2026-W32 - reports through 2026-08-05
1 new PDF(s). Ledger, inventory, workbook,
chart and the listing row-count high-water mark updated by the
scheduled run. Acceptance test passed before this commit was made.
</commit_message>
<xml_diff>
--- a/output/AMX_Buybacks.xlsx
+++ b/output/AMX_Buybacks.xlsx
@@ -15,7 +15,7 @@
     <sheet name="Chart" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Raw'!$A$1:$M$538</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Raw'!$A$1:$M$539</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Weekly'!$A$1:$P$199</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Monthly'!$A$1:$L$43</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Alerts'!$A$1:$E$6</definedName>
@@ -784,7 +784,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M538"/>
+  <dimension ref="A1:M539"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -26406,8 +26406,57 @@
       </c>
       <c r="M538" s="3" t="inlineStr"/>
     </row>
+    <row r="539">
+      <c r="A539" s="2" t="n">
+        <v>46239</v>
+      </c>
+      <c r="B539" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-05T17:13</t>
+        </is>
+      </c>
+      <c r="C539" s="3" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D539" s="3" t="inlineStr">
+        <is>
+          <t>INBUR</t>
+        </is>
+      </c>
+      <c r="E539" s="4" t="n">
+        <v>16802530840</v>
+      </c>
+      <c r="F539" s="4" t="n">
+        <v>16552980152</v>
+      </c>
+      <c r="G539" s="4" t="n">
+        <v>188000000</v>
+      </c>
+      <c r="H539" s="4" t="n">
+        <v>200000000</v>
+      </c>
+      <c r="I539" s="4" t="n">
+        <v>59982000000</v>
+      </c>
+      <c r="J539" s="4" t="n">
+        <v>59970000000</v>
+      </c>
+      <c r="K539" s="3" t="inlineStr">
+        <is>
+          <t>https://www.bmv.com.mx/docs-pub/recompra/recompra_1580281_1.pdf</t>
+        </is>
+      </c>
+      <c r="L539" s="3" t="inlineStr">
+        <is>
+          <t>505f90656a3945a5e7e63400551742db547383176235035c23685145b389c1a1</t>
+        </is>
+      </c>
+      <c r="M539" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M538"/>
+  <autoFilter ref="A1:M539"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -37941,13 +37990,13 @@
     </row>
     <row r="199">
       <c r="A199" s="2" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="B199" s="2" t="n">
         <v>46237</v>
       </c>
       <c r="C199" s="2" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="D199" s="3" t="inlineStr">
         <is>
@@ -37963,25 +38012,25 @@
         <v>46243</v>
       </c>
       <c r="G199" s="4" t="n">
-        <v>16802530840</v>
+        <v>16552980152</v>
       </c>
       <c r="H199" s="5" t="n">
-        <v>237578757</v>
+        <v>487129445</v>
       </c>
       <c r="I199" s="4" t="n">
-        <v>59982000000</v>
+        <v>59970000000</v>
       </c>
       <c r="J199" s="4" t="n">
-        <v>11000000</v>
+        <v>23000000</v>
       </c>
       <c r="K199" s="6" t="n">
-        <v>21.59806881818182</v>
+        <v>21.17954108695652</v>
       </c>
       <c r="L199" s="4" t="n">
         <v>0</v>
       </c>
       <c r="M199" s="7" t="n">
-        <v>0.0001833883498382848</v>
+        <v>0.000383525095881274</v>
       </c>
       <c r="N199" s="3" t="inlineStr">
         <is>
@@ -37989,11 +38038,11 @@
         </is>
       </c>
       <c r="O199" s="2" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="P199" s="3" t="inlineStr">
         <is>
-          <t>https://www.bmv.com.mx/docs-pub/recompra/recompra_1579878_1.pdf</t>
+          <t>https://www.bmv.com.mx/docs-pub/recompra/recompra_1580281_1.pdf</t>
         </is>
       </c>
     </row>
@@ -39886,35 +39935,35 @@
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="B43" s="4" t="n">
-        <v>16802530840</v>
+        <v>16552980152</v>
       </c>
       <c r="C43" s="5" t="n">
-        <v>237578757</v>
+        <v>487129445</v>
       </c>
       <c r="D43" s="4" t="n">
-        <v>59982000000</v>
+        <v>59970000000</v>
       </c>
       <c r="E43" s="4" t="n">
-        <v>11000000</v>
+        <v>23000000</v>
       </c>
       <c r="F43" s="6" t="n">
-        <v>21.59806881818182</v>
+        <v>21.17954108695652</v>
       </c>
       <c r="G43" s="4" t="n">
         <v>0</v>
       </c>
       <c r="H43" s="7" t="n">
-        <v>0.0001833883498382848</v>
+        <v>0.000383525095881274</v>
       </c>
       <c r="I43" s="2" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="J43" s="3" t="inlineStr">
         <is>
-          <t>https://www.bmv.com.mx/docs-pub/recompra/recompra_1579878_1.pdf</t>
+          <t>https://www.bmv.com.mx/docs-pub/recompra/recompra_1580281_1.pdf</t>
         </is>
       </c>
       <c r="K43" s="3" t="inlineStr">
@@ -39953,7 +40002,7 @@
     <row r="1">
       <c r="A1" s="8" t="inlineStr">
         <is>
-          <t>AMX Buybacks - 2026 YTD (through 04-Aug-2026)</t>
+          <t>AMX Buybacks - 2026 YTD (through 05-Aug-2026)</t>
         </is>
       </c>
     </row>
@@ -40124,16 +40173,16 @@
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>237578757</v>
+        <v>487129445</v>
       </c>
       <c r="C11" s="10" t="n">
-        <v>11000000</v>
+        <v>23000000</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>21.59806881818182</v>
+        <v>21.17954108695652</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>0.0001825317148854613</v>
+        <v>0.0003816572220332374</v>
       </c>
     </row>
     <row r="12">
@@ -40143,16 +40192,16 @@
         </is>
       </c>
       <c r="B12" s="12" t="n">
-        <v>6187559662</v>
+        <v>6437110350</v>
       </c>
       <c r="C12" s="13" t="n">
-        <v>281500000</v>
+        <v>293500000</v>
       </c>
       <c r="D12" s="14" t="n">
-        <v>21.98067375488455</v>
+        <v>21.932232879046</v>
       </c>
       <c r="E12" s="15" t="n">
-        <v>0.004671152521841579</v>
+        <v>0.004870278028989355</v>
       </c>
     </row>
   </sheetData>
@@ -40206,7 +40255,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>2026-08-05T23:03:08+00:00</t>
+          <t>2026-08-06T02:07:45+00:00</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -40233,7 +40282,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>2026-08-05T23:03:08+00:00</t>
+          <t>2026-08-06T02:07:45+00:00</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -40260,7 +40309,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>2026-08-05T23:03:08+00:00</t>
+          <t>2026-08-06T02:07:45+00:00</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -40287,7 +40336,7 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>2026-08-05T23:03:08+00:00</t>
+          <t>2026-08-06T02:07:45+00:00</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -40314,7 +40363,7 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>2026-08-05T23:03:08+00:00</t>
+          <t>2026-08-06T02:07:45+00:00</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Weekly run 2026-W32 - reports through 2026-08-07
1 new PDF(s). Ledger, inventory, workbook,
chart and the listing row-count high-water mark updated by the
scheduled run. Acceptance test passed before this commit was made.
</commit_message>
<xml_diff>
--- a/output/AMX_Buybacks.xlsx
+++ b/output/AMX_Buybacks.xlsx
@@ -15,7 +15,7 @@
     <sheet name="Chart" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Raw'!$A$1:$M$539</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Raw'!$A$1:$M$540</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Weekly'!$A$1:$P$199</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Monthly'!$A$1:$L$43</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Alerts'!$A$1:$E$6</definedName>
@@ -784,7 +784,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M539"/>
+  <dimension ref="A1:M540"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -26455,8 +26455,57 @@
       </c>
       <c r="M539" s="3" t="inlineStr"/>
     </row>
+    <row r="540">
+      <c r="A540" s="2" t="n">
+        <v>46241</v>
+      </c>
+      <c r="B540" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07T17:15</t>
+        </is>
+      </c>
+      <c r="C540" s="3" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D540" s="3" t="inlineStr">
+        <is>
+          <t>INBUR</t>
+        </is>
+      </c>
+      <c r="E540" s="4" t="n">
+        <v>16408304263</v>
+      </c>
+      <c r="F540" s="4" t="n">
+        <v>16285368061</v>
+      </c>
+      <c r="G540" s="4" t="n">
+        <v>207000000</v>
+      </c>
+      <c r="H540" s="4" t="n">
+        <v>213000000</v>
+      </c>
+      <c r="I540" s="4" t="n">
+        <v>59963000000</v>
+      </c>
+      <c r="J540" s="4" t="n">
+        <v>59957000000</v>
+      </c>
+      <c r="K540" s="3" t="inlineStr">
+        <is>
+          <t>https://www.bmv.com.mx/docs-pub/recompra/recompra_1581051_1.pdf</t>
+        </is>
+      </c>
+      <c r="L540" s="3" t="inlineStr">
+        <is>
+          <t>b098d9e99ef802218942852430e7cecd45836710b7a2a3999607e580e776e303</t>
+        </is>
+      </c>
+      <c r="M540" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M539"/>
+  <autoFilter ref="A1:M540"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -37990,13 +38039,13 @@
     </row>
     <row r="199">
       <c r="A199" s="2" t="n">
-        <v>46239</v>
+        <v>46241</v>
       </c>
       <c r="B199" s="2" t="n">
         <v>46237</v>
       </c>
       <c r="C199" s="2" t="n">
-        <v>46239</v>
+        <v>46241</v>
       </c>
       <c r="D199" s="3" t="inlineStr">
         <is>
@@ -38012,25 +38061,25 @@
         <v>46243</v>
       </c>
       <c r="G199" s="4" t="n">
-        <v>16552980152</v>
+        <v>16285368061</v>
       </c>
       <c r="H199" s="5" t="n">
-        <v>487129445</v>
+        <v>754741536</v>
       </c>
       <c r="I199" s="4" t="n">
-        <v>59970000000</v>
+        <v>59957000000</v>
       </c>
       <c r="J199" s="4" t="n">
-        <v>23000000</v>
+        <v>36000000</v>
       </c>
       <c r="K199" s="6" t="n">
-        <v>21.17954108695652</v>
+        <v>20.96504266666667</v>
       </c>
       <c r="L199" s="4" t="n">
         <v>0</v>
       </c>
       <c r="M199" s="7" t="n">
-        <v>0.000383525095881274</v>
+        <v>0.0006004303083876778</v>
       </c>
       <c r="N199" s="3" t="inlineStr">
         <is>
@@ -38038,11 +38087,11 @@
         </is>
       </c>
       <c r="O199" s="2" t="n">
-        <v>46239</v>
+        <v>46241</v>
       </c>
       <c r="P199" s="3" t="inlineStr">
         <is>
-          <t>https://www.bmv.com.mx/docs-pub/recompra/recompra_1580281_1.pdf</t>
+          <t>https://www.bmv.com.mx/docs-pub/recompra/recompra_1581051_1.pdf</t>
         </is>
       </c>
     </row>
@@ -39935,35 +39984,35 @@
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
-        <v>46239</v>
+        <v>46241</v>
       </c>
       <c r="B43" s="4" t="n">
-        <v>16552980152</v>
+        <v>16285368061</v>
       </c>
       <c r="C43" s="5" t="n">
-        <v>487129445</v>
+        <v>754741536</v>
       </c>
       <c r="D43" s="4" t="n">
-        <v>59970000000</v>
+        <v>59957000000</v>
       </c>
       <c r="E43" s="4" t="n">
-        <v>23000000</v>
+        <v>36000000</v>
       </c>
       <c r="F43" s="6" t="n">
-        <v>21.17954108695652</v>
+        <v>20.96504266666667</v>
       </c>
       <c r="G43" s="4" t="n">
         <v>0</v>
       </c>
       <c r="H43" s="7" t="n">
-        <v>0.000383525095881274</v>
+        <v>0.0006004303083876778</v>
       </c>
       <c r="I43" s="2" t="n">
-        <v>46239</v>
+        <v>46241</v>
       </c>
       <c r="J43" s="3" t="inlineStr">
         <is>
-          <t>https://www.bmv.com.mx/docs-pub/recompra/recompra_1580281_1.pdf</t>
+          <t>https://www.bmv.com.mx/docs-pub/recompra/recompra_1581051_1.pdf</t>
         </is>
       </c>
       <c r="K43" s="3" t="inlineStr">
@@ -40002,7 +40051,7 @@
     <row r="1">
       <c r="A1" s="8" t="inlineStr">
         <is>
-          <t>AMX Buybacks - 2026 YTD (through 05-Aug-2026)</t>
+          <t>AMX Buybacks - 2026 YTD (through 07-Aug-2026)</t>
         </is>
       </c>
     </row>
@@ -40173,16 +40222,16 @@
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>487129445</v>
+        <v>754741536</v>
       </c>
       <c r="C11" s="10" t="n">
-        <v>23000000</v>
+        <v>36000000</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>21.17954108695652</v>
+        <v>20.96504266666667</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>0.0003816572220332374</v>
+        <v>0.000597376521443328</v>
       </c>
     </row>
     <row r="12">
@@ -40192,16 +40241,16 @@
         </is>
       </c>
       <c r="B12" s="12" t="n">
-        <v>6437110350</v>
+        <v>6704722441</v>
       </c>
       <c r="C12" s="13" t="n">
-        <v>293500000</v>
+        <v>306500000</v>
       </c>
       <c r="D12" s="14" t="n">
-        <v>21.932232879046</v>
+        <v>21.875114</v>
       </c>
       <c r="E12" s="15" t="n">
-        <v>0.004870278028989355</v>
+        <v>0.005085997328399446</v>
       </c>
     </row>
   </sheetData>
@@ -40255,7 +40304,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>2026-08-06T02:07:45+00:00</t>
+          <t>2026-08-08T03:01:39+00:00</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -40282,7 +40331,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>2026-08-06T02:07:45+00:00</t>
+          <t>2026-08-08T03:01:39+00:00</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -40309,7 +40358,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>2026-08-06T02:07:45+00:00</t>
+          <t>2026-08-08T03:01:39+00:00</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -40336,7 +40385,7 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>2026-08-06T02:07:45+00:00</t>
+          <t>2026-08-08T03:01:39+00:00</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -40363,7 +40412,7 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>2026-08-06T02:07:45+00:00</t>
+          <t>2026-08-08T03:01:39+00:00</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Weekly run 2026-W33 - reports through 2026-08-14
1 new PDF(s). Ledger, inventory, workbook,
chart and the listing row-count high-water mark updated by the
scheduled run. Acceptance test passed before this commit was made.
</commit_message>
<xml_diff>
--- a/output/AMX_Buybacks.xlsx
+++ b/output/AMX_Buybacks.xlsx
@@ -15,8 +15,8 @@
     <sheet name="Chart" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Raw'!$A$1:$M$540</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Weekly'!$A$1:$P$199</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Raw'!$A$1:$M$541</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Weekly'!$A$1:$P$200</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Monthly'!$A$1:$L$43</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Alerts'!$A$1:$E$6</definedName>
   </definedNames>
@@ -784,7 +784,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M540"/>
+  <dimension ref="A1:M541"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -26504,8 +26504,57 @@
       </c>
       <c r="M540" s="3" t="inlineStr"/>
     </row>
+    <row r="541">
+      <c r="A541" s="2" t="n">
+        <v>46248</v>
+      </c>
+      <c r="B541" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-14T17:20</t>
+        </is>
+      </c>
+      <c r="C541" s="3" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D541" s="3" t="inlineStr">
+        <is>
+          <t>INBUR</t>
+        </is>
+      </c>
+      <c r="E541" s="4" t="n">
+        <v>15604902698</v>
+      </c>
+      <c r="F541" s="4" t="n">
+        <v>15524623835</v>
+      </c>
+      <c r="G541" s="4" t="n">
+        <v>247000000</v>
+      </c>
+      <c r="H541" s="4" t="n">
+        <v>251000000</v>
+      </c>
+      <c r="I541" s="4" t="n">
+        <v>59923000000</v>
+      </c>
+      <c r="J541" s="4" t="n">
+        <v>59919000000</v>
+      </c>
+      <c r="K541" s="3" t="inlineStr">
+        <is>
+          <t>https://www.bmv.com.mx/docs-pub/recompra/recompra_1582524_1.pdf</t>
+        </is>
+      </c>
+      <c r="L541" s="3" t="inlineStr">
+        <is>
+          <t>8dde826e59921713cbd1cca7715aa5f5be7c092393de346bf239e3c7efbb84df</t>
+        </is>
+      </c>
+      <c r="M541" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M540"/>
+  <autoFilter ref="A1:M541"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -26516,7 +26565,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P199"/>
+  <dimension ref="A1:P200"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -38049,7 +38098,7 @@
       </c>
       <c r="D199" s="3" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="E199" s="3" t="inlineStr">
@@ -38095,8 +38144,66 @@
         </is>
       </c>
     </row>
+    <row r="200">
+      <c r="A200" s="2" t="n">
+        <v>46248</v>
+      </c>
+      <c r="B200" s="2" t="n">
+        <v>46248</v>
+      </c>
+      <c r="C200" s="2" t="n">
+        <v>46248</v>
+      </c>
+      <c r="D200" s="3" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="E200" s="3" t="inlineStr">
+        <is>
+          <t>2026-W33</t>
+        </is>
+      </c>
+      <c r="F200" s="2" t="n">
+        <v>46250</v>
+      </c>
+      <c r="G200" s="4" t="n">
+        <v>15524623835</v>
+      </c>
+      <c r="H200" s="5" t="n">
+        <v>760744226</v>
+      </c>
+      <c r="I200" s="4" t="n">
+        <v>59919000000</v>
+      </c>
+      <c r="J200" s="4" t="n">
+        <v>38000000</v>
+      </c>
+      <c r="K200" s="6" t="n">
+        <v>20.01958489473684</v>
+      </c>
+      <c r="L200" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M200" s="7" t="n">
+        <v>0.0006341894891436773</v>
+      </c>
+      <c r="N200" s="3" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O200" s="2" t="n">
+        <v>46248</v>
+      </c>
+      <c r="P200" s="3" t="inlineStr">
+        <is>
+          <t>https://www.bmv.com.mx/docs-pub/recompra/recompra_1582524_1.pdf</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:P199"/>
+  <autoFilter ref="A1:P200"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -39984,35 +40091,35 @@
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
-        <v>46241</v>
+        <v>46248</v>
       </c>
       <c r="B43" s="4" t="n">
-        <v>16285368061</v>
+        <v>15524623835</v>
       </c>
       <c r="C43" s="5" t="n">
-        <v>754741536</v>
+        <v>1515485762</v>
       </c>
       <c r="D43" s="4" t="n">
-        <v>59957000000</v>
+        <v>59919000000</v>
       </c>
       <c r="E43" s="4" t="n">
-        <v>36000000</v>
+        <v>74000000</v>
       </c>
       <c r="F43" s="6" t="n">
-        <v>20.96504266666667</v>
+        <v>20.47953732432432</v>
       </c>
       <c r="G43" s="4" t="n">
         <v>0</v>
       </c>
       <c r="H43" s="7" t="n">
-        <v>0.0006004303083876778</v>
+        <v>0.001235000584121898</v>
       </c>
       <c r="I43" s="2" t="n">
-        <v>46241</v>
+        <v>46248</v>
       </c>
       <c r="J43" s="3" t="inlineStr">
         <is>
-          <t>https://www.bmv.com.mx/docs-pub/recompra/recompra_1581051_1.pdf</t>
+          <t>https://www.bmv.com.mx/docs-pub/recompra/recompra_1582524_1.pdf</t>
         </is>
       </c>
       <c r="K43" s="3" t="inlineStr">
@@ -40051,7 +40158,7 @@
     <row r="1">
       <c r="A1" s="8" t="inlineStr">
         <is>
-          <t>AMX Buybacks - 2026 YTD (through 07-Aug-2026)</t>
+          <t>AMX Buybacks - 2026 YTD (through 14-Aug-2026)</t>
         </is>
       </c>
     </row>
@@ -40222,16 +40329,16 @@
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>754741536</v>
+        <v>1515485762</v>
       </c>
       <c r="C11" s="10" t="n">
-        <v>36000000</v>
+        <v>74000000</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>20.96504266666667</v>
+        <v>20.47953732432432</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>0.000597376521443328</v>
+        <v>0.001227940627411286</v>
       </c>
     </row>
     <row r="12">
@@ -40241,16 +40348,16 @@
         </is>
       </c>
       <c r="B12" s="12" t="n">
-        <v>6704722441</v>
+        <v>7465466667</v>
       </c>
       <c r="C12" s="13" t="n">
-        <v>306500000</v>
+        <v>344500000</v>
       </c>
       <c r="D12" s="14" t="n">
-        <v>21.875114</v>
+        <v>21.67044025253991</v>
       </c>
       <c r="E12" s="15" t="n">
-        <v>0.005085997328399446</v>
+        <v>0.005716561434367403</v>
       </c>
     </row>
   </sheetData>
@@ -40304,7 +40411,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>2026-08-08T03:01:39+00:00</t>
+          <t>2026-08-15T02:19:55+00:00</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -40331,7 +40438,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>2026-08-08T03:01:39+00:00</t>
+          <t>2026-08-15T02:19:55+00:00</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -40358,7 +40465,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>2026-08-08T03:01:39+00:00</t>
+          <t>2026-08-15T02:19:55+00:00</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -40385,7 +40492,7 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>2026-08-08T03:01:39+00:00</t>
+          <t>2026-08-15T02:19:55+00:00</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -40412,7 +40519,7 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>2026-08-08T03:01:39+00:00</t>
+          <t>2026-08-15T02:19:55+00:00</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Weekly run 2026-W34 - reports through 2026-08-21
1 new PDF(s). Ledger, inventory, workbook,
chart and the listing row-count high-water mark updated by the
scheduled run. Acceptance test passed before this commit was made.
</commit_message>
<xml_diff>
--- a/output/AMX_Buybacks.xlsx
+++ b/output/AMX_Buybacks.xlsx
@@ -15,8 +15,8 @@
     <sheet name="Chart" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Raw'!$A$1:$M$541</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Weekly'!$A$1:$P$200</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Raw'!$A$1:$M$542</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Weekly'!$A$1:$P$201</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Monthly'!$A$1:$L$43</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Alerts'!$A$1:$E$6</definedName>
   </definedNames>
@@ -784,7 +784,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M541"/>
+  <dimension ref="A1:M542"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -26553,8 +26553,57 @@
       </c>
       <c r="M541" s="3" t="inlineStr"/>
     </row>
+    <row r="542">
+      <c r="A542" s="2" t="n">
+        <v>46255</v>
+      </c>
+      <c r="B542" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-21T17:29</t>
+        </is>
+      </c>
+      <c r="C542" s="3" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D542" s="3" t="inlineStr">
+        <is>
+          <t>INBUR</t>
+        </is>
+      </c>
+      <c r="E542" s="4" t="n">
+        <v>15444677856</v>
+      </c>
+      <c r="F542" s="4" t="n">
+        <v>15416619084</v>
+      </c>
+      <c r="G542" s="4" t="n">
+        <v>255000000</v>
+      </c>
+      <c r="H542" s="4" t="n">
+        <v>256400000</v>
+      </c>
+      <c r="I542" s="4" t="n">
+        <v>59915000000</v>
+      </c>
+      <c r="J542" s="4" t="n">
+        <v>59913600000</v>
+      </c>
+      <c r="K542" s="3" t="inlineStr">
+        <is>
+          <t>https://www.bmv.com.mx/docs-pub/recompra/recompra_1583826_1.pdf</t>
+        </is>
+      </c>
+      <c r="L542" s="3" t="inlineStr">
+        <is>
+          <t>ad02cc63bf930d30f250ede587fd7f4ee65465aeb5516763c67826156acd2dfb</t>
+        </is>
+      </c>
+      <c r="M542" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M541"/>
+  <autoFilter ref="A1:M542"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -26565,7 +26614,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P200"/>
+  <dimension ref="A1:P201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -38156,7 +38205,7 @@
       </c>
       <c r="D200" s="3" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="E200" s="3" t="inlineStr">
@@ -38202,8 +38251,66 @@
         </is>
       </c>
     </row>
+    <row r="201">
+      <c r="A201" s="2" t="n">
+        <v>46255</v>
+      </c>
+      <c r="B201" s="2" t="n">
+        <v>46255</v>
+      </c>
+      <c r="C201" s="2" t="n">
+        <v>46255</v>
+      </c>
+      <c r="D201" s="3" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="E201" s="3" t="inlineStr">
+        <is>
+          <t>2026-W34</t>
+        </is>
+      </c>
+      <c r="F201" s="2" t="n">
+        <v>46257</v>
+      </c>
+      <c r="G201" s="4" t="n">
+        <v>15416619084</v>
+      </c>
+      <c r="H201" s="5" t="n">
+        <v>108004751</v>
+      </c>
+      <c r="I201" s="4" t="n">
+        <v>59913600000</v>
+      </c>
+      <c r="J201" s="4" t="n">
+        <v>5400000</v>
+      </c>
+      <c r="K201" s="6" t="n">
+        <v>20.00087981481482</v>
+      </c>
+      <c r="L201" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M201" s="7" t="n">
+        <v>9.01297868931261e-05</v>
+      </c>
+      <c r="N201" s="3" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O201" s="2" t="n">
+        <v>46255</v>
+      </c>
+      <c r="P201" s="3" t="inlineStr">
+        <is>
+          <t>https://www.bmv.com.mx/docs-pub/recompra/recompra_1583826_1.pdf</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:P200"/>
+  <autoFilter ref="A1:P201"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -40091,35 +40198,35 @@
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
-        <v>46248</v>
+        <v>46255</v>
       </c>
       <c r="B43" s="4" t="n">
-        <v>15524623835</v>
+        <v>15416619084</v>
       </c>
       <c r="C43" s="5" t="n">
-        <v>1515485762</v>
+        <v>1623490513</v>
       </c>
       <c r="D43" s="4" t="n">
-        <v>59919000000</v>
+        <v>59913600000</v>
       </c>
       <c r="E43" s="4" t="n">
-        <v>74000000</v>
+        <v>79400000</v>
       </c>
       <c r="F43" s="6" t="n">
-        <v>20.47953732432432</v>
+        <v>20.44698379093199</v>
       </c>
       <c r="G43" s="4" t="n">
         <v>0</v>
       </c>
       <c r="H43" s="7" t="n">
-        <v>0.001235000584121898</v>
+        <v>0.001325241681354484</v>
       </c>
       <c r="I43" s="2" t="n">
-        <v>46248</v>
+        <v>46255</v>
       </c>
       <c r="J43" s="3" t="inlineStr">
         <is>
-          <t>https://www.bmv.com.mx/docs-pub/recompra/recompra_1582524_1.pdf</t>
+          <t>https://www.bmv.com.mx/docs-pub/recompra/recompra_1583826_1.pdf</t>
         </is>
       </c>
       <c r="K43" s="3" t="inlineStr">
@@ -40158,7 +40265,7 @@
     <row r="1">
       <c r="A1" s="8" t="inlineStr">
         <is>
-          <t>AMX Buybacks - 2026 YTD (through 14-Aug-2026)</t>
+          <t>AMX Buybacks - 2026 YTD (through 21-Aug-2026)</t>
         </is>
       </c>
     </row>
@@ -40329,16 +40436,16 @@
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>1515485762</v>
+        <v>1623490513</v>
       </c>
       <c r="C11" s="10" t="n">
-        <v>74000000</v>
+        <v>79400000</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>20.47953732432432</v>
+        <v>20.44698379093199</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>0.001227940627411286</v>
+        <v>0.001317547105627785</v>
       </c>
     </row>
     <row r="12">
@@ -40348,16 +40455,16 @@
         </is>
       </c>
       <c r="B12" s="12" t="n">
-        <v>7465466667</v>
+        <v>7573471418</v>
       </c>
       <c r="C12" s="13" t="n">
-        <v>344500000</v>
+        <v>349900000</v>
       </c>
       <c r="D12" s="14" t="n">
-        <v>21.67044025253991</v>
+        <v>21.64467395827379</v>
       </c>
       <c r="E12" s="15" t="n">
-        <v>0.005716561434367403</v>
+        <v>0.005806167912583903</v>
       </c>
     </row>
   </sheetData>
@@ -40411,7 +40518,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>2026-08-15T02:19:55+00:00</t>
+          <t>2026-08-22T02:29:38+00:00</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -40438,7 +40545,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>2026-08-15T02:19:55+00:00</t>
+          <t>2026-08-22T02:29:38+00:00</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -40465,7 +40572,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>2026-08-15T02:19:55+00:00</t>
+          <t>2026-08-22T02:29:38+00:00</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -40492,7 +40599,7 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>2026-08-15T02:19:55+00:00</t>
+          <t>2026-08-22T02:29:38+00:00</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -40519,7 +40626,7 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>2026-08-15T02:19:55+00:00</t>
+          <t>2026-08-22T02:29:38+00:00</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Weekly run 2026-W35 - reports through 2026-08-28
1 new PDF(s). Ledger, inventory, workbook,
chart and the listing row-count high-water mark updated by the
scheduled run. Acceptance test passed before this commit was made.
</commit_message>
<xml_diff>
--- a/output/AMX_Buybacks.xlsx
+++ b/output/AMX_Buybacks.xlsx
@@ -15,8 +15,8 @@
     <sheet name="Chart" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Raw'!$A$1:$M$542</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Weekly'!$A$1:$P$201</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Raw'!$A$1:$M$543</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Weekly'!$A$1:$P$202</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Monthly'!$A$1:$L$43</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Alerts'!$A$1:$E$6</definedName>
   </definedNames>
@@ -784,7 +784,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M542"/>
+  <dimension ref="A1:M543"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -26602,8 +26602,57 @@
       </c>
       <c r="M542" s="3" t="inlineStr"/>
     </row>
+    <row r="543">
+      <c r="A543" s="2" t="n">
+        <v>46262</v>
+      </c>
+      <c r="B543" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-28T16:39</t>
+        </is>
+      </c>
+      <c r="C543" s="3" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D543" s="3" t="inlineStr">
+        <is>
+          <t>INBUR</t>
+        </is>
+      </c>
+      <c r="E543" s="4" t="n">
+        <v>15274361103</v>
+      </c>
+      <c r="F543" s="4" t="n">
+        <v>15175448691</v>
+      </c>
+      <c r="G543" s="4" t="n">
+        <v>263500000</v>
+      </c>
+      <c r="H543" s="4" t="n">
+        <v>268500000</v>
+      </c>
+      <c r="I543" s="4" t="n">
+        <v>59906500000</v>
+      </c>
+      <c r="J543" s="4" t="n">
+        <v>59901500000</v>
+      </c>
+      <c r="K543" s="3" t="inlineStr">
+        <is>
+          <t>https://www.bmv.com.mx/docs-pub/recompra/recompra_1585332_1.pdf</t>
+        </is>
+      </c>
+      <c r="L543" s="3" t="inlineStr">
+        <is>
+          <t>aed9c09f3f325d1b42f4f1adc745182b0b4f1de15d7e6e81bf933d910c9b8cb7</t>
+        </is>
+      </c>
+      <c r="M543" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M542"/>
+  <autoFilter ref="A1:M543"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -26614,7 +26663,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P201"/>
+  <dimension ref="A1:P202"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -38263,7 +38312,7 @@
       </c>
       <c r="D201" s="3" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="E201" s="3" t="inlineStr">
@@ -38309,8 +38358,66 @@
         </is>
       </c>
     </row>
+    <row r="202">
+      <c r="A202" s="2" t="n">
+        <v>46262</v>
+      </c>
+      <c r="B202" s="2" t="n">
+        <v>46262</v>
+      </c>
+      <c r="C202" s="2" t="n">
+        <v>46262</v>
+      </c>
+      <c r="D202" s="3" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="E202" s="3" t="inlineStr">
+        <is>
+          <t>2026-W35</t>
+        </is>
+      </c>
+      <c r="F202" s="2" t="n">
+        <v>46264</v>
+      </c>
+      <c r="G202" s="4" t="n">
+        <v>15175448691</v>
+      </c>
+      <c r="H202" s="5" t="n">
+        <v>241170393</v>
+      </c>
+      <c r="I202" s="4" t="n">
+        <v>59901500000</v>
+      </c>
+      <c r="J202" s="4" t="n">
+        <v>12100000</v>
+      </c>
+      <c r="K202" s="6" t="n">
+        <v>19.93143743801653</v>
+      </c>
+      <c r="L202" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M202" s="7" t="n">
+        <v>0.0002019982805105047</v>
+      </c>
+      <c r="N202" s="3" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O202" s="2" t="n">
+        <v>46262</v>
+      </c>
+      <c r="P202" s="3" t="inlineStr">
+        <is>
+          <t>https://www.bmv.com.mx/docs-pub/recompra/recompra_1585332_1.pdf</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:P201"/>
+  <autoFilter ref="A1:P202"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -40198,35 +40305,35 @@
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
-        <v>46255</v>
+        <v>46262</v>
       </c>
       <c r="B43" s="4" t="n">
-        <v>15416619084</v>
+        <v>15175448691</v>
       </c>
       <c r="C43" s="5" t="n">
-        <v>1623490513</v>
+        <v>1864660906</v>
       </c>
       <c r="D43" s="4" t="n">
-        <v>59913600000</v>
+        <v>59901500000</v>
       </c>
       <c r="E43" s="4" t="n">
-        <v>79400000</v>
+        <v>91500000</v>
       </c>
       <c r="F43" s="6" t="n">
-        <v>20.44698379093199</v>
+        <v>20.378807715847</v>
       </c>
       <c r="G43" s="4" t="n">
         <v>0</v>
       </c>
       <c r="H43" s="7" t="n">
-        <v>0.001325241681354484</v>
+        <v>0.001527507658405883</v>
       </c>
       <c r="I43" s="2" t="n">
-        <v>46255</v>
+        <v>46262</v>
       </c>
       <c r="J43" s="3" t="inlineStr">
         <is>
-          <t>https://www.bmv.com.mx/docs-pub/recompra/recompra_1583826_1.pdf</t>
+          <t>https://www.bmv.com.mx/docs-pub/recompra/recompra_1585332_1.pdf</t>
         </is>
       </c>
       <c r="K43" s="3" t="inlineStr">
@@ -40265,7 +40372,7 @@
     <row r="1">
       <c r="A1" s="8" t="inlineStr">
         <is>
-          <t>AMX Buybacks - 2026 YTD (through 21-Aug-2026)</t>
+          <t>AMX Buybacks - 2026 YTD (through 28-Aug-2026)</t>
         </is>
       </c>
     </row>
@@ -40436,16 +40543,16 @@
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>1623490513</v>
+        <v>1864660906</v>
       </c>
       <c r="C11" s="10" t="n">
-        <v>79400000</v>
+        <v>91500000</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>20.44698379093199</v>
+        <v>20.378807715847</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>0.001317547105627785</v>
+        <v>0.001518331992001792</v>
       </c>
     </row>
     <row r="12">
@@ -40455,16 +40562,16 @@
         </is>
       </c>
       <c r="B12" s="12" t="n">
-        <v>7573471418</v>
+        <v>7814641811</v>
       </c>
       <c r="C12" s="13" t="n">
-        <v>349900000</v>
+        <v>362000000</v>
       </c>
       <c r="D12" s="14" t="n">
-        <v>21.64467395827379</v>
+        <v>21.58740831767956</v>
       </c>
       <c r="E12" s="15" t="n">
-        <v>0.005806167912583903</v>
+        <v>0.00600695279895791</v>
       </c>
     </row>
   </sheetData>
@@ -40518,7 +40625,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>2026-08-22T02:29:38+00:00</t>
+          <t>2026-08-29T07:54:02+00:00</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -40545,7 +40652,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>2026-08-22T02:29:38+00:00</t>
+          <t>2026-08-29T07:54:02+00:00</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -40572,7 +40679,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>2026-08-22T02:29:38+00:00</t>
+          <t>2026-08-29T07:54:02+00:00</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -40599,7 +40706,7 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>2026-08-22T02:29:38+00:00</t>
+          <t>2026-08-29T07:54:02+00:00</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -40626,7 +40733,7 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>2026-08-22T02:29:38+00:00</t>
+          <t>2026-08-29T07:54:02+00:00</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Weekly run 2026-W36 - reports through 2026-09-04
2 new PDF(s). Ledger, inventory, workbook,
chart and the listing row-count high-water mark updated by the
scheduled run. Acceptance test passed before this commit was made.
</commit_message>
<xml_diff>
--- a/output/AMX_Buybacks.xlsx
+++ b/output/AMX_Buybacks.xlsx
@@ -15,9 +15,9 @@
     <sheet name="Chart" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Raw'!$A$1:$M$543</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Weekly'!$A$1:$P$202</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Monthly'!$A$1:$L$43</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Raw'!$A$1:$M$545</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Weekly'!$A$1:$P$204</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Monthly'!$A$1:$L$44</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Alerts'!$A$1:$E$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -208,12 +208,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Monthly'!$K$3:$K$43</f>
+              <f>'Monthly'!$K$3:$K$44</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Monthly'!$C$3:$C$43</f>
+              <f>'Monthly'!$C$3:$C$44</f>
             </numRef>
           </val>
         </ser>
@@ -254,7 +254,7 @@
           </marker>
           <val>
             <numRef>
-              <f>'Monthly'!$H$3:$H$43</f>
+              <f>'Monthly'!$H$3:$H$44</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -784,7 +784,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M543"/>
+  <dimension ref="A1:M545"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -26651,8 +26651,106 @@
       </c>
       <c r="M543" s="3" t="inlineStr"/>
     </row>
+    <row r="544">
+      <c r="A544" s="2" t="n">
+        <v>46265</v>
+      </c>
+      <c r="B544" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-31T17:32</t>
+        </is>
+      </c>
+      <c r="C544" s="3" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D544" s="3" t="inlineStr">
+        <is>
+          <t>INBUR</t>
+        </is>
+      </c>
+      <c r="E544" s="4" t="n">
+        <v>15175448691</v>
+      </c>
+      <c r="F544" s="4" t="n">
+        <v>15126294893</v>
+      </c>
+      <c r="G544" s="4" t="n">
+        <v>268500000</v>
+      </c>
+      <c r="H544" s="4" t="n">
+        <v>271000000</v>
+      </c>
+      <c r="I544" s="4" t="n">
+        <v>59901500000</v>
+      </c>
+      <c r="J544" s="4" t="n">
+        <v>59899000000</v>
+      </c>
+      <c r="K544" s="3" t="inlineStr">
+        <is>
+          <t>https://www.bmv.com.mx/docs-pub/recompra/recompra_1585645_1.pdf</t>
+        </is>
+      </c>
+      <c r="L544" s="3" t="inlineStr">
+        <is>
+          <t>f3c4feafdbc915941933aea939d7d43fb919158b324d4c0e45dfca19a05570eb</t>
+        </is>
+      </c>
+      <c r="M544" s="3" t="inlineStr"/>
+    </row>
+    <row r="545">
+      <c r="A545" s="2" t="n">
+        <v>46269</v>
+      </c>
+      <c r="B545" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-04T17:09</t>
+        </is>
+      </c>
+      <c r="C545" s="3" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D545" s="3" t="inlineStr">
+        <is>
+          <t>INBUR</t>
+        </is>
+      </c>
+      <c r="E545" s="4" t="n">
+        <v>14633950121</v>
+      </c>
+      <c r="F545" s="4" t="n">
+        <v>13855735685</v>
+      </c>
+      <c r="G545" s="4" t="n">
+        <v>296300000</v>
+      </c>
+      <c r="H545" s="4" t="n">
+        <v>336300000</v>
+      </c>
+      <c r="I545" s="4" t="n">
+        <v>59873700000</v>
+      </c>
+      <c r="J545" s="4" t="n">
+        <v>59833700000</v>
+      </c>
+      <c r="K545" s="3" t="inlineStr">
+        <is>
+          <t>https://www.bmv.com.mx/docs-pub/recompra/recompra_1587051_1.pdf</t>
+        </is>
+      </c>
+      <c r="L545" s="3" t="inlineStr">
+        <is>
+          <t>469a86754cdc76437f5eb47af7a57b43da0e50421e75c4b8594895b82547ac31</t>
+        </is>
+      </c>
+      <c r="M545" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M543"/>
+  <autoFilter ref="A1:M545"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -26663,7 +26761,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P202"/>
+  <dimension ref="A1:P204"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -38370,7 +38468,7 @@
       </c>
       <c r="D202" s="3" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="E202" s="3" t="inlineStr">
@@ -38416,8 +38514,124 @@
         </is>
       </c>
     </row>
+    <row r="203">
+      <c r="A203" s="2" t="n">
+        <v>46265</v>
+      </c>
+      <c r="B203" s="2" t="n">
+        <v>46265</v>
+      </c>
+      <c r="C203" s="2" t="n">
+        <v>46265</v>
+      </c>
+      <c r="D203" s="3" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="E203" s="3" t="inlineStr">
+        <is>
+          <t>2026-W36</t>
+        </is>
+      </c>
+      <c r="F203" s="2" t="n">
+        <v>46271</v>
+      </c>
+      <c r="G203" s="4" t="n">
+        <v>15126294893</v>
+      </c>
+      <c r="H203" s="5" t="n">
+        <v>49153798</v>
+      </c>
+      <c r="I203" s="4" t="n">
+        <v>59899000000</v>
+      </c>
+      <c r="J203" s="4" t="n">
+        <v>2500000</v>
+      </c>
+      <c r="K203" s="6" t="n">
+        <v>19.6615192</v>
+      </c>
+      <c r="L203" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M203" s="7" t="n">
+        <v>4.173692382176664e-05</v>
+      </c>
+      <c r="N203" s="3" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O203" s="2" t="n">
+        <v>46265</v>
+      </c>
+      <c r="P203" s="3" t="inlineStr">
+        <is>
+          <t>https://www.bmv.com.mx/docs-pub/recompra/recompra_1585645_1.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="2" t="n">
+        <v>46269</v>
+      </c>
+      <c r="B204" s="2" t="n">
+        <v>46269</v>
+      </c>
+      <c r="C204" s="2" t="n">
+        <v>46269</v>
+      </c>
+      <c r="D204" s="3" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="E204" s="3" t="inlineStr">
+        <is>
+          <t>2026-W36</t>
+        </is>
+      </c>
+      <c r="F204" s="2" t="n">
+        <v>46271</v>
+      </c>
+      <c r="G204" s="4" t="n">
+        <v>13855735685</v>
+      </c>
+      <c r="H204" s="5" t="n">
+        <v>1270559208</v>
+      </c>
+      <c r="I204" s="4" t="n">
+        <v>59833700000</v>
+      </c>
+      <c r="J204" s="4" t="n">
+        <v>65300000</v>
+      </c>
+      <c r="K204" s="6" t="n">
+        <v>19.45726199081164</v>
+      </c>
+      <c r="L204" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M204" s="7" t="n">
+        <v>0.001091358214517906</v>
+      </c>
+      <c r="N204" s="3" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O204" s="2" t="n">
+        <v>46269</v>
+      </c>
+      <c r="P204" s="3" t="inlineStr">
+        <is>
+          <t>https://www.bmv.com.mx/docs-pub/recompra/recompra_1587051_1.pdf</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:P202"/>
+  <autoFilter ref="A1:P204"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -38428,7 +38642,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L43"/>
+  <dimension ref="A1:L44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -40305,35 +40519,35 @@
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
-        <v>46262</v>
+        <v>46265</v>
       </c>
       <c r="B43" s="4" t="n">
-        <v>15175448691</v>
+        <v>15126294893</v>
       </c>
       <c r="C43" s="5" t="n">
-        <v>1864660906</v>
+        <v>1913814704</v>
       </c>
       <c r="D43" s="4" t="n">
-        <v>59901500000</v>
+        <v>59899000000</v>
       </c>
       <c r="E43" s="4" t="n">
-        <v>91500000</v>
+        <v>94000000</v>
       </c>
       <c r="F43" s="6" t="n">
-        <v>20.378807715847</v>
+        <v>20.35973089361702</v>
       </c>
       <c r="G43" s="4" t="n">
         <v>0</v>
       </c>
       <c r="H43" s="7" t="n">
-        <v>0.001527507658405883</v>
+        <v>0.001569308335698426</v>
       </c>
       <c r="I43" s="2" t="n">
-        <v>46262</v>
+        <v>46265</v>
       </c>
       <c r="J43" s="3" t="inlineStr">
         <is>
-          <t>https://www.bmv.com.mx/docs-pub/recompra/recompra_1585332_1.pdf</t>
+          <t>https://www.bmv.com.mx/docs-pub/recompra/recompra_1585645_1.pdf</t>
         </is>
       </c>
       <c r="K43" s="3" t="inlineStr">
@@ -40347,8 +40561,52 @@
         </is>
       </c>
     </row>
+    <row r="44">
+      <c r="A44" s="2" t="n">
+        <v>46269</v>
+      </c>
+      <c r="B44" s="4" t="n">
+        <v>13855735685</v>
+      </c>
+      <c r="C44" s="5" t="n">
+        <v>1270559208</v>
+      </c>
+      <c r="D44" s="4" t="n">
+        <v>59833700000</v>
+      </c>
+      <c r="E44" s="4" t="n">
+        <v>65300000</v>
+      </c>
+      <c r="F44" s="6" t="n">
+        <v>19.45726199081164</v>
+      </c>
+      <c r="G44" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H44" s="7" t="n">
+        <v>0.001091358214517906</v>
+      </c>
+      <c r="I44" s="2" t="n">
+        <v>46269</v>
+      </c>
+      <c r="J44" s="3" t="inlineStr">
+        <is>
+          <t>https://www.bmv.com.mx/docs-pub/recompra/recompra_1587051_1.pdf</t>
+        </is>
+      </c>
+      <c r="K44" s="3" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="L44" s="3" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L43"/>
+  <autoFilter ref="A1:L44"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -40359,7 +40617,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -40372,7 +40630,7 @@
     <row r="1">
       <c r="A1" s="8" t="inlineStr">
         <is>
-          <t>AMX Buybacks - 2026 YTD (through 28-Aug-2026)</t>
+          <t>AMX Buybacks - 2026 YTD (through 04-Sep-2026)</t>
         </is>
       </c>
     </row>
@@ -40543,35 +40801,54 @@
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>1864660906</v>
+        <v>1913814704</v>
       </c>
       <c r="C11" s="10" t="n">
-        <v>91500000</v>
+        <v>94000000</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>20.378807715847</v>
+        <v>20.35973089361702</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>0.001518331992001792</v>
+        <v>0.001559816472657579</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="11" t="inlineStr">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>1270559208</v>
+      </c>
+      <c r="C12" s="10" t="n">
+        <v>65300000</v>
+      </c>
+      <c r="D12" s="6" t="n">
+        <v>19.45726199081164</v>
+      </c>
+      <c r="E12" s="7" t="n">
+        <v>0.001083574634729148</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="11" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B12" s="12" t="n">
-        <v>7814641811</v>
-      </c>
-      <c r="C12" s="13" t="n">
-        <v>362000000</v>
-      </c>
-      <c r="D12" s="14" t="n">
-        <v>21.58740831767956</v>
-      </c>
-      <c r="E12" s="15" t="n">
-        <v>0.00600695279895791</v>
+      <c r="B13" s="12" t="n">
+        <v>9134354817</v>
+      </c>
+      <c r="C13" s="13" t="n">
+        <v>429800000</v>
+      </c>
+      <c r="D13" s="14" t="n">
+        <v>21.25257053745928</v>
+      </c>
+      <c r="E13" s="15" t="n">
+        <v>0.007132011914342844</v>
       </c>
     </row>
   </sheetData>
@@ -40625,7 +40902,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>2026-08-29T07:54:02+00:00</t>
+          <t>2026-09-05T05:47:20+00:00</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -40652,7 +40929,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>2026-08-29T07:54:02+00:00</t>
+          <t>2026-09-05T05:47:20+00:00</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -40679,7 +40956,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>2026-08-29T07:54:02+00:00</t>
+          <t>2026-09-05T05:47:20+00:00</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -40706,7 +40983,7 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>2026-08-29T07:54:02+00:00</t>
+          <t>2026-09-05T05:47:20+00:00</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -40733,7 +41010,7 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>2026-08-29T07:54:02+00:00</t>
+          <t>2026-09-05T05:47:20+00:00</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">

</xml_diff>